<commit_message>
v0.2: calibrated US pass-through beta, OU Monte Carlo, vulnerability ranking
- Empirically calibrate US crude-to-pump beta (0.36, R2=0.51) replacing v0 guess,
  update Excel model with the real value
- src/monte_carlo.py: OU calibration on Brent (2010-on) and 10k-path 12-month
  simulation run through the same margin logic as the Excel ShockEngine sheet
- 3 charts: Brent history with OU mean, Monte Carlo fan chart, vulnerability
  ranking bar chart (Brazil 42pct breach probability vs US ~0pct)
- Notebook fully executed end to end, real outputs committed, zero errors
- India/China/Germany/Brazil pass-through and the CapitalIQ screen remain open,
  documented in README and notebook section 6

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/fuel_shock_model.xlsx
+++ b/excel/fuel_shock_model.xlsx
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>0.9</v>
+        <v>0.36</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>0.5</v>
@@ -701,7 +701,7 @@
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>v0 estimate of tax wedge. Calibrate by regressing pump on crude, 2015 to 2025</t>
+          <t>US CALIBRATED (regression of 13-week pct moves, Brent vs EIA diesel, 1994-2026, R2=0.51, beta=0.36; 2015-on subset gives 0.33). Other four still v0 estimates, calibrate with Eurostat/PPAC/NDRC/ANP or Bloomberg</t>
         </is>
       </c>
     </row>

</xml_diff>